<commit_message>
Simplify Power Budget page and workbook
Template sections A-E only, short notes. Adds back the 2.5V reference divider load (428.250mA with margin).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WMeTzg44UYnfGmciHkCZq2
</commit_message>
<xml_diff>
--- a/docs/05-Power-Budget/Fill-A-Bot-Main-Control-Power-Budget.xlsx
+++ b/docs/05-Power-Budget/Fill-A-Bot-Main-Control-Power-Budget.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="203">
   <si>
     <t xml:space="preserve">Main Control Board Power Budget</t>
   </si>
@@ -82,7 +82,7 @@
     <t xml:space="preserve">Derived ceiling</t>
   </si>
   <si>
-    <t xml:space="preserve">Microchip gives a maximum IDD only at VDD = 3.0V (Table 47-2: 8.2mA at 64MHz HFINTOSC). There is no 5V maximum. Ceiling: the PIC may not dissipate more than 800mW, so its own supply current is at most 800mW / 4.9V = 163.3mA (my PIC pins sink the LED and pull-up currents; they barely source anything). Add the 5.5mA Nano allowance = 168.8mA, rounded up to 170mA. This is not a datasheet operating current.</t>
+    <t xml:space="preserve">Microchip only lists max current at 3V, not 5V. Safe estimate: 800mW max power / 4.9V = 163.3mA, plus 5.5mA for the Nano LED and level shifters, rounded up to 170mA.</t>
   </si>
   <si>
     <t xml:space="preserve">https://ww1.microchip.com/downloads/aemDocuments/documents/MCU08/ProductDocuments/DataSheets/PIC18F27-47-57Q43-Microcontroller-Data-Sheet-XLP-DS40002147.pdf</t>
@@ -100,7 +100,7 @@
     <t xml:space="preserve">Datasheet max + calculated</t>
   </si>
   <si>
-    <t xml:space="preserve">2 x 0.170mA IQ max (guaranteed at 25C) + 5.1V / 9.9k ohm = 0.515mA, a bound on the current U3A or U3B can push through Rin and Rf. The +/-30mA supply-pin figure is an absolute-maximum stress rating, not a current the part uses, so it is not used.</t>
+    <t xml:space="preserve">2 x 0.170mA max per op amp + 5.1V / 9.9k ohm through the feedback resistors.</t>
   </si>
   <si>
     <t xml:space="preserve">https://ww1.microchip.com/downloads/en/DeviceDoc/MCP6001-1R-1U-2-4-1-MHz-Low-Power-Op-Amp-DS20001733L.pdf</t>
@@ -118,7 +118,7 @@
     <t xml:space="preserve">Datasheet max</t>
   </si>
   <si>
-    <t xml:space="preserve">Electrical Characteristics: IDD 3.0mA max at VDD = 5.0V (typ 1.0mA). Counted once. No separate driver IC.</t>
+    <t xml:space="preserve">IDD 3.0mA max at 5.0V.</t>
   </si>
   <si>
     <t xml:space="preserve">https://newhavendisplay.com/content/specs/NHD-0216K1Z-FL-YBW.pdf</t>
@@ -130,7 +130,7 @@
     <t xml:space="preserve">4.9 to 5.1V; 5V used</t>
   </si>
   <si>
-    <t xml:space="preserve">Electrical Characteristics: ILED 156mA max at VLED = 5.0V (typ 130mA), built-in resistor. The rail can reach 5.1V; the 25% margin covers the small extra current.</t>
+    <t xml:space="preserve">Backlight 156mA max at 5.0V.</t>
   </si>
   <si>
     <t xml:space="preserve">LDR cup-sensor divider</t>
@@ -145,7 +145,7 @@
     <t xml:space="preserve">Calculated bound</t>
   </si>
   <si>
-    <t xml:space="preserve">5.1V / 9.9k ohm = 0.515mA even if the LDR went to 0 ohm. The datasheet gives resistance and power, not a supply current.</t>
+    <t xml:space="preserve">5.1V / 9.9k ohm, worst case if the LDR goes to 0 ohm.</t>
   </si>
   <si>
     <t xml:space="preserve">https://media.digikey.com/pdf/data%20sheets/photonic%20detetectors%20inc%20pdfs/pdv-p8103.pdf</t>
@@ -154,7 +154,7 @@
     <t xml:space="preserve">Major-component subtotal</t>
   </si>
   <si>
-    <t xml:space="preserve">Value types: Datasheet max = guaranteed limit from the manufacturer's electrical table. Calculated bound = Ohm's law with the rail at 5.1V and the resistor at its minimum value. Derived ceiling = built from an absolute-maximum rating because no 5V operating maximum is published. Typical values are listed only for comparison and are not used in the totals.</t>
+    <t xml:space="preserve">Resistor currents use the worst case: 5.1V rail and each resistor at its lowest value.</t>
   </si>
   <si>
     <t xml:space="preserve">B. 5V rail: every load assigned once, then one 25% safety margin</t>
@@ -163,15 +163,24 @@
     <t xml:space="preserve">Same as Section A.</t>
   </si>
   <si>
+    <t xml:space="preserve">2.5V reference divider for U3B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Two 10k ohm, 1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.1V / 19.8k ohm = 0.258mA.</t>
+  </si>
+  <si>
     <t xml:space="preserve">LCD E pull-down (while E is high)</t>
   </si>
   <si>
     <t xml:space="preserve">100k ohm</t>
   </si>
   <si>
-    <t xml:space="preserve">5V</t>
-  </si>
-  <si>
     <t xml:space="preserve">5.1V / 99k ohm = 0.052mA. Sourced by RC5.</t>
   </si>
   <si>
@@ -490,7 +499,7 @@
     <t xml:space="preserve">Keep the sink away from the LCD (rated to 70C).</t>
   </si>
   <si>
-    <t xml:space="preserve">Notes: (1) The 3.0V PIC IDD table is not a guaranteed maximum at 5.0V, so the 170mA Nano entry is a derived ceiling, not a datasheet operating current. (2) Stress ratings (PIC 350mA VSS pin, MCP6002 +/-30mA) are not used as operating currents. (3) The LCD values are specified at 5.0V and 25C. (4) Real current, plug fit, cup detection, and enclosure temperature still need prototype measurements.</t>
+    <t xml:space="preserve">Note: the real board current and regulator temperature still need to be measured on the built board.</t>
   </si>
   <si>
     <t xml:space="preserve">Inputs used by the formulas above</t>
@@ -553,7 +562,7 @@
     <t xml:space="preserve">Selected value</t>
   </si>
   <si>
-    <t xml:space="preserve">LDR divider R1, four button pull-ups, and U3B Rin are all 10k ohm, 1%.</t>
+    <t xml:space="preserve">LDR divider R1, the two reference divider resistors, four button pull-ups, and U3B Rin are all 10k ohm, 1%.</t>
   </si>
   <si>
     <t xml:space="preserve">Fixed resistor tolerance</t>
@@ -1701,12 +1710,12 @@
         <v>1</v>
       </c>
       <c r="F24" s="7" t="n">
-        <f aca="false">ROUNDUP($G$72/($G$113*(1-$G$105))*1000,3)</f>
-        <v>0.052</v>
+        <f aca="false">ROUNDUP($G$72/(2*$G$104*(1-$G$105))*1000,3)</f>
+        <v>0.258</v>
       </c>
       <c r="G24" s="7" t="n">
         <f aca="false">E24*F24</f>
-        <v>0.052</v>
+        <v>0.258</v>
       </c>
       <c r="H24" s="5" t="s">
         <v>18</v>
@@ -1732,12 +1741,12 @@
         <v>1</v>
       </c>
       <c r="F25" s="7" t="n">
-        <f aca="false">ROUNDUP($G$72/($G$106*(1-$G$107))*1000,3)</f>
-        <v>0.638</v>
+        <f aca="false">ROUNDUP($G$72/($G$113*(1-$G$105))*1000,3)</f>
+        <v>0.052</v>
       </c>
       <c r="G25" s="7" t="n">
         <f aca="false">E25*F25</f>
-        <v>0.638</v>
+        <v>0.052</v>
       </c>
       <c r="H25" s="5" t="s">
         <v>18</v>
@@ -1763,12 +1772,12 @@
         <v>1</v>
       </c>
       <c r="F26" s="7" t="n">
-        <f aca="false">$G$109*ROUNDUP($G$72/($G$108*(1-$G$105))*1000,3)</f>
-        <v>7.026</v>
+        <f aca="false">ROUNDUP($G$72/($G$106*(1-$G$107))*1000,3)</f>
+        <v>0.638</v>
       </c>
       <c r="G26" s="7" t="n">
         <f aca="false">E26*F26</f>
-        <v>7.026</v>
+        <v>0.638</v>
       </c>
       <c r="H26" s="5" t="s">
         <v>18</v>
@@ -1794,12 +1803,12 @@
         <v>1</v>
       </c>
       <c r="F27" s="7" t="n">
-        <f aca="false">ROUNDUP($G$110*$G$72/($G$104*(1-$G$105))*1000,3)</f>
-        <v>2.061</v>
+        <f aca="false">$G$109*ROUNDUP($G$72/($G$108*(1-$G$105))*1000,3)</f>
+        <v>7.026</v>
       </c>
       <c r="G27" s="7" t="n">
         <f aca="false">E27*F27</f>
-        <v>2.061</v>
+        <v>7.026</v>
       </c>
       <c r="H27" s="5" t="s">
         <v>18</v>
@@ -1825,352 +1834,367 @@
         <v>1</v>
       </c>
       <c r="F28" s="7" t="n">
+        <f aca="false">ROUNDUP($G$110*$G$72/($G$104*(1-$G$105))*1000,3)</f>
+        <v>2.061</v>
+      </c>
+      <c r="G28" s="7" t="n">
+        <f aca="false">E28*F28</f>
+        <v>2.061</v>
+      </c>
+      <c r="H28" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I28" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="J28" s="8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B29" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E29" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="7" t="n">
         <f aca="false">ROUNDUP($G$112*$G$72/($G$111*(1-$G$105))*1000,3)</f>
         <v>2.193</v>
       </c>
-      <c r="G28" s="7" t="n">
-        <f aca="false">E28*F28</f>
+      <c r="G29" s="7" t="n">
+        <f aca="false">E29*F29</f>
         <v>2.193</v>
       </c>
-      <c r="H28" s="5" t="s">
+      <c r="H29" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="I28" s="5" t="s">
+      <c r="I29" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="J28" s="8" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="C29" s="15"/>
-      <c r="D29" s="15"/>
-      <c r="E29" s="15"/>
-      <c r="F29" s="15"/>
-      <c r="G29" s="11" t="n">
-        <f aca="false">SUM(G19:G28)</f>
-        <v>342.342</v>
-      </c>
-      <c r="H29" s="16" t="s">
+      <c r="J29" s="8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B30" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="C30" s="15"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="15"/>
+      <c r="F30" s="15"/>
+      <c r="G30" s="11" t="n">
+        <f aca="false">SUM(G19:G29)</f>
+        <v>342.6</v>
+      </c>
+      <c r="H30" s="16" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="17" t="n">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B31" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2"/>
+      <c r="G31" s="17" t="n">
         <v>0.25</v>
       </c>
-      <c r="H30" s="16"/>
-      <c r="J30" s="16" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="15" t="s">
-        <v>66</v>
-      </c>
-      <c r="C31" s="15"/>
-      <c r="D31" s="15"/>
-      <c r="E31" s="15"/>
-      <c r="F31" s="15"/>
-      <c r="G31" s="11" t="n">
-        <f aca="false">ROUNDUP(G29*(1+G30),3)</f>
-        <v>427.928</v>
-      </c>
-      <c r="H31" s="16" t="s">
+      <c r="H31" s="16"/>
+      <c r="J31" s="16" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B32" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="C32" s="15"/>
+      <c r="D32" s="15"/>
+      <c r="E32" s="15"/>
+      <c r="F32" s="15"/>
+      <c r="G32" s="11" t="n">
+        <f aca="false">ROUNDUP(G30*(1+G31),3)</f>
+        <v>428.25</v>
+      </c>
+      <c r="H32" s="16" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
-      <c r="F32" s="2"/>
-      <c r="G32" s="18" t="n">
-        <f aca="false">G31*$G$70/1000</f>
-        <v>2.13964</v>
-      </c>
-      <c r="H32" s="16" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B34" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="C34" s="3"/>
-      <c r="D34" s="3"/>
-      <c r="E34" s="3"/>
-      <c r="F34" s="3"/>
-      <c r="G34" s="3"/>
-      <c r="H34" s="3"/>
-      <c r="I34" s="3"/>
-      <c r="J34" s="3"/>
-      <c r="K34" s="3"/>
-    </row>
-    <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B35" s="4" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B33" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="18" t="n">
+        <f aca="false">G32*$G$70/1000</f>
+        <v>2.14125</v>
+      </c>
+      <c r="H33" s="16" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B35" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C35" s="3"/>
+      <c r="D35" s="3"/>
+      <c r="E35" s="3"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3"/>
+      <c r="H35" s="3"/>
+      <c r="I35" s="3"/>
+      <c r="J35" s="3"/>
+      <c r="K35" s="3"/>
+    </row>
+    <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B36" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C35" s="4" t="s">
+      <c r="C36" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D35" s="4" t="s">
+      <c r="D36" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="E35" s="4" t="s">
+      <c r="E36" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="F35" s="4" t="s">
+      <c r="F36" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G35" s="4" t="s">
+      <c r="G36" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="H35" s="4" t="s">
+      <c r="H36" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="I35" s="4" t="s">
+      <c r="I36" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="J35" s="4" t="s">
+      <c r="J36" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="K35" s="4" t="s">
+      <c r="K36" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="C36" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="D36" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="E36" s="6" t="n">
+    <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B37" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D37" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="E37" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F36" s="9" t="n">
+      <c r="F37" s="9" t="n">
         <v>1500</v>
       </c>
-      <c r="G36" s="7" t="n">
-        <f aca="false">E36*F36</f>
+      <c r="G37" s="7" t="n">
+        <f aca="false">E37*F37</f>
         <v>1500</v>
       </c>
-      <c r="H36" s="5" t="s">
+      <c r="H37" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="I36" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="J36" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="K36" s="8" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="2" t="s">
+      <c r="I37" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2"/>
-      <c r="F37" s="2"/>
-      <c r="G37" s="18" t="n">
-        <f aca="false">G31</f>
-        <v>427.928</v>
-      </c>
-      <c r="H37" s="16" t="s">
-        <v>18</v>
+      <c r="J37" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="K37" s="8" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B38" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="C38" s="15"/>
-      <c r="D38" s="15"/>
-      <c r="E38" s="15"/>
-      <c r="F38" s="15"/>
-      <c r="G38" s="11" t="n">
-        <f aca="false">G36-G37</f>
-        <v>1072.072</v>
+      <c r="B38" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C38" s="2"/>
+      <c r="D38" s="2"/>
+      <c r="E38" s="2"/>
+      <c r="F38" s="2"/>
+      <c r="G38" s="18" t="n">
+        <f aca="false">G32</f>
+        <v>428.25</v>
       </c>
       <c r="H38" s="16" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B39" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
-      <c r="F39" s="2"/>
-      <c r="G39" s="18" t="n">
+      <c r="B39" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="C39" s="15"/>
+      <c r="D39" s="15"/>
+      <c r="E39" s="15"/>
+      <c r="F39" s="15"/>
+      <c r="G39" s="11" t="n">
+        <f aca="false">G37-G38</f>
+        <v>1071.75</v>
+      </c>
+      <c r="H39" s="16" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B40" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="2"/>
+      <c r="F40" s="2"/>
+      <c r="G40" s="18" t="n">
         <f aca="false">$G$88</f>
         <v>1220</v>
       </c>
-      <c r="H39" s="16" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B40" s="15" t="s">
-        <v>79</v>
-      </c>
-      <c r="C40" s="15"/>
-      <c r="D40" s="15"/>
-      <c r="E40" s="15"/>
-      <c r="F40" s="15"/>
-      <c r="G40" s="11" t="n">
-        <f aca="false">G39-G31</f>
-        <v>792.072</v>
-      </c>
       <c r="H40" s="16" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B42" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="C42" s="3"/>
-      <c r="D42" s="3"/>
-      <c r="E42" s="3"/>
-      <c r="F42" s="3"/>
-      <c r="G42" s="3"/>
-      <c r="H42" s="3"/>
-      <c r="I42" s="3"/>
-      <c r="J42" s="3"/>
-      <c r="K42" s="3"/>
-    </row>
-    <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B43" s="4" t="s">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B41" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="C41" s="15"/>
+      <c r="D41" s="15"/>
+      <c r="E41" s="15"/>
+      <c r="F41" s="15"/>
+      <c r="G41" s="11" t="n">
+        <f aca="false">G40-G32</f>
+        <v>791.75</v>
+      </c>
+      <c r="H41" s="16" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B43" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C43" s="3"/>
+      <c r="D43" s="3"/>
+      <c r="E43" s="3"/>
+      <c r="F43" s="3"/>
+      <c r="G43" s="3"/>
+      <c r="H43" s="3"/>
+      <c r="I43" s="3"/>
+      <c r="J43" s="3"/>
+      <c r="K43" s="3"/>
+    </row>
+    <row r="44" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B44" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C43" s="4" t="s">
+      <c r="C44" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D43" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="E43" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="F43" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="G43" s="4" t="s">
+      <c r="D44" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="H43" s="4" t="s">
+      <c r="E44" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="F44" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="G44" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H44" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="I43" s="4" t="s">
+      <c r="I44" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="J43" s="4" t="s">
+      <c r="J44" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="K43" s="4" t="s">
+      <c r="K44" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B44" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="C44" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="D44" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="E44" s="6" t="n">
+    <row r="45" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B45" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="E45" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="F44" s="9" t="n">
+      <c r="F45" s="9" t="n">
         <v>2000</v>
       </c>
-      <c r="G44" s="7" t="n">
-        <f aca="false">F44</f>
+      <c r="G45" s="7" t="n">
+        <f aca="false">F45</f>
         <v>2000</v>
       </c>
-      <c r="H44" s="5" t="s">
+      <c r="H45" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="I44" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="J44" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="K44" s="8" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B45" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
-      <c r="E45" s="2"/>
-      <c r="F45" s="2"/>
-      <c r="G45" s="18" t="n">
-        <f aca="false">G36</f>
+      <c r="I45" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="J45" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="K45" s="8" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B46" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C46" s="2"/>
+      <c r="D46" s="2"/>
+      <c r="E46" s="2"/>
+      <c r="F46" s="2"/>
+      <c r="G46" s="18" t="n">
+        <f aca="false">G37</f>
         <v>1500</v>
-      </c>
-      <c r="H45" s="16" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B46" s="15" t="s">
-        <v>91</v>
-      </c>
-      <c r="C46" s="15"/>
-      <c r="D46" s="15"/>
-      <c r="E46" s="15"/>
-      <c r="F46" s="15"/>
-      <c r="G46" s="11" t="n">
-        <f aca="false">G44-G45</f>
-        <v>500</v>
       </c>
       <c r="H46" s="16" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B47" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="C47" s="2"/>
-      <c r="D47" s="2"/>
-      <c r="E47" s="2"/>
-      <c r="F47" s="2"/>
-      <c r="G47" s="18" t="n">
-        <f aca="false">G31</f>
-        <v>427.928</v>
+      <c r="B47" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="C47" s="15"/>
+      <c r="D47" s="15"/>
+      <c r="E47" s="15"/>
+      <c r="F47" s="15"/>
+      <c r="G47" s="11" t="n">
+        <f aca="false">G45-G46</f>
+        <v>500</v>
       </c>
       <c r="H47" s="16" t="s">
         <v>18</v>
@@ -2178,105 +2202,105 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B48" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
       <c r="E48" s="2"/>
       <c r="F48" s="2"/>
-      <c r="G48" s="19" t="n">
-        <v>10</v>
+      <c r="G48" s="18" t="n">
+        <f aca="false">G32</f>
+        <v>428.25</v>
       </c>
       <c r="H48" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="I48" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="J48" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="K48" s="16" t="s">
-        <v>75</v>
-      </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B49" s="15" t="s">
-        <v>95</v>
-      </c>
-      <c r="C49" s="15"/>
-      <c r="D49" s="15"/>
-      <c r="E49" s="15"/>
-      <c r="F49" s="15"/>
-      <c r="G49" s="11" t="n">
-        <f aca="false">G47+G48</f>
-        <v>437.928</v>
+      <c r="B49" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C49" s="2"/>
+      <c r="D49" s="2"/>
+      <c r="E49" s="2"/>
+      <c r="F49" s="2"/>
+      <c r="G49" s="19" t="n">
+        <v>10</v>
       </c>
       <c r="H49" s="16" t="s">
         <v>18</v>
       </c>
+      <c r="I49" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="J49" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="K49" s="16" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B50" s="15" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C50" s="15"/>
       <c r="D50" s="15"/>
       <c r="E50" s="15"/>
       <c r="F50" s="15"/>
       <c r="G50" s="11" t="n">
-        <f aca="false">G44-G49</f>
-        <v>1562.072</v>
+        <f aca="false">G48+G49</f>
+        <v>438.25</v>
       </c>
       <c r="H50" s="16" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B51" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="C51" s="2"/>
-      <c r="D51" s="2"/>
-      <c r="E51" s="2"/>
-      <c r="F51" s="2"/>
-      <c r="G51" s="18" t="n">
-        <f aca="false">E44*G49/1000</f>
-        <v>3.941352</v>
+      <c r="B51" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="C51" s="15"/>
+      <c r="D51" s="15"/>
+      <c r="E51" s="15"/>
+      <c r="F51" s="15"/>
+      <c r="G51" s="11" t="n">
+        <f aca="false">G45-G50</f>
+        <v>1561.75</v>
       </c>
       <c r="H51" s="16" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B53" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="C53" s="3"/>
-      <c r="D53" s="3"/>
-      <c r="E53" s="3"/>
-      <c r="F53" s="3"/>
-      <c r="G53" s="3"/>
-      <c r="H53" s="3"/>
-      <c r="I53" s="3"/>
-      <c r="J53" s="3"/>
-      <c r="K53" s="3"/>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B54" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="C54" s="2"/>
-      <c r="D54" s="2"/>
-      <c r="E54" s="2"/>
-      <c r="F54" s="2"/>
-      <c r="G54" s="8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B52" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="H54" s="16"/>
-      <c r="J54" s="16" t="s">
+      <c r="C52" s="2"/>
+      <c r="D52" s="2"/>
+      <c r="E52" s="2"/>
+      <c r="F52" s="2"/>
+      <c r="G52" s="18" t="n">
+        <f aca="false">E45*G50/1000</f>
+        <v>3.94425</v>
+      </c>
+      <c r="H52" s="16" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B54" s="3" t="s">
         <v>101</v>
       </c>
+      <c r="C54" s="3"/>
+      <c r="D54" s="3"/>
+      <c r="E54" s="3"/>
+      <c r="F54" s="3"/>
+      <c r="G54" s="3"/>
+      <c r="H54" s="3"/>
+      <c r="I54" s="3"/>
+      <c r="J54" s="3"/>
+      <c r="K54" s="3"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B55" s="2" t="s">
@@ -2287,26 +2311,42 @@
       <c r="E55" s="2"/>
       <c r="F55" s="2"/>
       <c r="G55" s="8" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="H55" s="16"/>
+      <c r="J55" s="16" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B56" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" s="2"/>
       <c r="E56" s="2"/>
       <c r="F56" s="2"/>
       <c r="G56" s="8" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="H56" s="16"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B57" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C57" s="2"/>
+      <c r="D57" s="2"/>
+      <c r="E57" s="2"/>
+      <c r="F57" s="2"/>
+      <c r="G57" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="H57" s="16"/>
     </row>
     <row r="64" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B64" s="3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C64" s="3"/>
       <c r="D64" s="3"/>
@@ -2320,7 +2360,7 @@
     </row>
     <row r="65" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B65" s="3" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C65" s="3"/>
       <c r="D65" s="3"/>
@@ -2334,23 +2374,23 @@
     </row>
     <row r="66" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B66" s="2" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C66" s="2"/>
       <c r="D66" s="2"/>
       <c r="E66" s="2"/>
       <c r="F66" s="2"/>
       <c r="G66" s="18" t="n">
-        <f aca="false">E44</f>
+        <f aca="false">E45</f>
         <v>9</v>
       </c>
       <c r="H66" s="16" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B67" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" s="2"/>
@@ -2364,15 +2404,15 @@
         <v>31</v>
       </c>
       <c r="J67" s="16" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K67" s="16" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B68" s="2" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" s="2"/>
@@ -2383,12 +2423,12 @@
         <v>9.45</v>
       </c>
       <c r="H68" s="16" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B69" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" s="2"/>
@@ -2399,12 +2439,12 @@
         <v>8.55</v>
       </c>
       <c r="H69" s="16" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B70" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" s="2"/>
@@ -2414,21 +2454,21 @@
         <v>5</v>
       </c>
       <c r="H70" s="16" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="I70" s="16" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="J70" s="16" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="K70" s="16" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B71" s="2" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C71" s="2"/>
       <c r="D71" s="2"/>
@@ -2438,21 +2478,21 @@
         <v>4.9</v>
       </c>
       <c r="H71" s="16" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="I71" s="16" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="J71" s="16" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="K71" s="16" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B72" s="2" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" s="2"/>
@@ -2462,21 +2502,21 @@
         <v>5.1</v>
       </c>
       <c r="H72" s="16" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="I72" s="16" t="s">
         <v>31</v>
       </c>
       <c r="J72" s="16" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="K72" s="16" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B73" s="2" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C73" s="2"/>
       <c r="D73" s="2"/>
@@ -2486,21 +2526,21 @@
         <v>0.15</v>
       </c>
       <c r="H73" s="16" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="I73" s="16" t="s">
         <v>31</v>
       </c>
       <c r="J73" s="16" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="K73" s="16" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B74" s="2" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="C74" s="2"/>
       <c r="D74" s="2"/>
@@ -2510,40 +2550,40 @@
         <v>1.5</v>
       </c>
       <c r="H74" s="16" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="I74" s="16" t="s">
         <v>31</v>
       </c>
       <c r="J74" s="16" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="K74" s="16" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B75" s="2" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C75" s="2"/>
       <c r="D75" s="2"/>
       <c r="E75" s="2"/>
       <c r="F75" s="2"/>
       <c r="G75" s="18" t="n">
-        <f aca="false">G69-G73/2-$G$114*G49/1000</f>
-        <v>8.408434944</v>
+        <f aca="false">G69-G73/2-$G$114*G50/1000</f>
+        <v>8.408386</v>
       </c>
       <c r="H75" s="16" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="I75" s="16" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B76" s="2" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C76" s="2"/>
       <c r="D76" s="2"/>
@@ -2554,18 +2594,18 @@
         <v>6.6</v>
       </c>
       <c r="H76" s="16" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="I76" s="16" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="J76" s="16" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B77" s="15" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C77" s="15"/>
       <c r="D77" s="15"/>
@@ -2573,21 +2613,21 @@
       <c r="F77" s="15"/>
       <c r="G77" s="11" t="n">
         <f aca="false">G75-G76</f>
-        <v>1.808434944</v>
+        <v>1.808386</v>
       </c>
       <c r="H77" s="16" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="I77" s="16" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="J77" s="16" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B78" s="3" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C78" s="3"/>
       <c r="D78" s="3"/>
@@ -2601,7 +2641,7 @@
     </row>
     <row r="79" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B79" s="2" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C79" s="2"/>
       <c r="D79" s="2"/>
@@ -2611,18 +2651,18 @@
         <v>40</v>
       </c>
       <c r="H79" s="16" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="I79" s="16" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="J79" s="16" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B80" s="2" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C80" s="2"/>
       <c r="D80" s="2"/>
@@ -2632,21 +2672,21 @@
         <v>4</v>
       </c>
       <c r="H80" s="16" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="I80" s="16" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="J80" s="16" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="K80" s="16" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B81" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C81" s="2"/>
       <c r="D81" s="2"/>
@@ -2656,21 +2696,21 @@
         <v>1</v>
       </c>
       <c r="H81" s="16" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="I81" s="16" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="J81" s="16" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="K81" s="16" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B82" s="2" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C82" s="2"/>
       <c r="D82" s="2"/>
@@ -2680,21 +2720,21 @@
         <v>10</v>
       </c>
       <c r="H82" s="16" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="I82" s="16" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="J82" s="16" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="K82" s="16" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B83" s="2" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="C83" s="2"/>
       <c r="D83" s="2"/>
@@ -2705,15 +2745,15 @@
         <v>15</v>
       </c>
       <c r="H83" s="16" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="I83" s="16" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B84" s="2" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C84" s="2"/>
       <c r="D84" s="2"/>
@@ -2723,21 +2763,21 @@
         <v>125</v>
       </c>
       <c r="H84" s="16" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="I84" s="16" t="s">
         <v>31</v>
       </c>
       <c r="J84" s="16" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="K84" s="16" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B85" s="2" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="C85" s="2"/>
       <c r="D85" s="2"/>
@@ -2748,34 +2788,34 @@
         <v>5.66666666666667</v>
       </c>
       <c r="H85" s="16" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="I85" s="16" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B86" s="2" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="C86" s="2"/>
       <c r="D86" s="2"/>
       <c r="E86" s="2"/>
       <c r="F86" s="2"/>
       <c r="G86" s="18" t="n">
-        <f aca="false">(G68-G71)*G31/1000+G68*G48/1000</f>
-        <v>2.0415724</v>
+        <f aca="false">(G68-G71)*G32/1000+G68*G49/1000</f>
+        <v>2.0430375</v>
       </c>
       <c r="H86" s="16" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="I86" s="16" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B87" s="15" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C87" s="15"/>
       <c r="D87" s="15"/>
@@ -2783,40 +2823,40 @@
       <c r="F87" s="15"/>
       <c r="G87" s="22" t="n">
         <f aca="false">G79+G86*G83</f>
-        <v>70.623586</v>
+        <v>70.6455625</v>
       </c>
       <c r="H87" s="16" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="I87" s="16" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B88" s="2" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="C88" s="2"/>
       <c r="D88" s="2"/>
       <c r="E88" s="2"/>
       <c r="F88" s="2"/>
       <c r="G88" s="18" t="n">
-        <f aca="false">ROUNDDOWN((G85-G68*G48/1000)/(G68-G71)*1000,-1)</f>
+        <f aca="false">ROUNDDOWN((G85-G68*G49/1000)/(G68-G71)*1000,-1)</f>
         <v>1220</v>
       </c>
       <c r="H88" s="16" t="s">
         <v>18</v>
       </c>
       <c r="I88" s="16" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="J88" s="16" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B89" s="15" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="C89" s="15"/>
       <c r="D89" s="15"/>
@@ -2824,18 +2864,18 @@
       <c r="F89" s="15"/>
       <c r="G89" s="22" t="n">
         <f aca="false">G84-G87</f>
-        <v>54.376414</v>
+        <v>54.3544375</v>
       </c>
       <c r="H89" s="16" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="I89" s="16" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B90" s="2" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="C90" s="2"/>
       <c r="D90" s="2"/>
@@ -2843,21 +2883,21 @@
       <c r="F90" s="2"/>
       <c r="G90" s="21" t="n">
         <f aca="false">G86*G82</f>
-        <v>20.415724</v>
+        <v>20.430375</v>
       </c>
       <c r="H90" s="16" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="I90" s="16" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="J90" s="16" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="92" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B92" s="13" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="C92" s="13"/>
       <c r="D92" s="13"/>
@@ -2871,7 +2911,7 @@
     </row>
     <row r="98" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B98" s="3" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C98" s="3"/>
       <c r="D98" s="3"/>
@@ -2885,14 +2925,14 @@
     </row>
     <row r="99" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B99" s="4" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C99" s="4"/>
       <c r="D99" s="4"/>
       <c r="E99" s="4"/>
       <c r="F99" s="4"/>
       <c r="G99" s="4" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="H99" s="4" t="s">
         <v>11</v>
@@ -2909,7 +2949,7 @@
     </row>
     <row r="100" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B100" s="2" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="C100" s="2"/>
       <c r="D100" s="2"/>
@@ -2919,13 +2959,13 @@
         <v>800</v>
       </c>
       <c r="H100" s="16" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I100" s="16" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="J100" s="16" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="K100" s="16" t="s">
         <v>21</v>
@@ -2933,7 +2973,7 @@
     </row>
     <row r="101" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B101" s="2" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="C101" s="2"/>
       <c r="D101" s="2"/>
@@ -2946,18 +2986,18 @@
         <v>18</v>
       </c>
       <c r="I101" s="16" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="J101" s="16" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="K101" s="16" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B102" s="2" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C102" s="2"/>
       <c r="D102" s="2"/>
@@ -2973,7 +3013,7 @@
         <v>31</v>
       </c>
       <c r="J102" s="16" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="K102" s="16" t="s">
         <v>27</v>
@@ -2981,7 +3021,7 @@
     </row>
     <row r="103" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B103" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C103" s="2"/>
       <c r="D103" s="2"/>
@@ -2991,19 +3031,19 @@
         <v>2</v>
       </c>
       <c r="H103" s="16" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="I103" s="16" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="J103" s="16" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="K103" s="16"/>
     </row>
     <row r="104" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B104" s="2" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="C104" s="2"/>
       <c r="D104" s="2"/>
@@ -3013,19 +3053,19 @@
         <v>10000</v>
       </c>
       <c r="H104" s="16" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="I104" s="16" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="J104" s="16" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="K104" s="16"/>
     </row>
     <row r="105" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B105" s="2" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="C105" s="2"/>
       <c r="D105" s="2"/>
@@ -3036,16 +3076,16 @@
       </c>
       <c r="H105" s="16"/>
       <c r="I105" s="16" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="J105" s="16" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="K105" s="16"/>
     </row>
     <row r="106" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B106" s="2" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="C106" s="2"/>
       <c r="D106" s="2"/>
@@ -3055,19 +3095,19 @@
         <v>10000</v>
       </c>
       <c r="H106" s="16" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="I106" s="16" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="J106" s="16" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="K106" s="16"/>
     </row>
     <row r="107" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B107" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="C107" s="2"/>
       <c r="D107" s="2"/>
@@ -3078,16 +3118,16 @@
       </c>
       <c r="H107" s="16"/>
       <c r="I107" s="16" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="J107" s="16" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="K107" s="16"/>
     </row>
     <row r="108" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B108" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="C108" s="2"/>
       <c r="D108" s="2"/>
@@ -3097,19 +3137,19 @@
         <v>2200</v>
       </c>
       <c r="H108" s="16" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="I108" s="16" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="J108" s="16" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="K108" s="16"/>
     </row>
     <row r="109" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B109" s="2" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C109" s="2"/>
       <c r="D109" s="2"/>
@@ -3119,19 +3159,19 @@
         <v>3</v>
       </c>
       <c r="H109" s="16" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="I109" s="16" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="J109" s="16" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="K109" s="16"/>
     </row>
     <row r="110" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B110" s="2" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="C110" s="2"/>
       <c r="D110" s="2"/>
@@ -3141,19 +3181,19 @@
         <v>4</v>
       </c>
       <c r="H110" s="16" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="I110" s="16" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="J110" s="16" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="K110" s="16"/>
     </row>
     <row r="111" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B111" s="2" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="C111" s="2"/>
       <c r="D111" s="2"/>
@@ -3163,19 +3203,19 @@
         <v>4700</v>
       </c>
       <c r="H111" s="16" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="I111" s="16" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="J111" s="16" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="K111" s="16"/>
     </row>
     <row r="112" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B112" s="2" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="C112" s="2"/>
       <c r="D112" s="2"/>
@@ -3185,19 +3225,19 @@
         <v>2</v>
       </c>
       <c r="H112" s="16" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="I112" s="16" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="J112" s="16" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="K112" s="16"/>
     </row>
     <row r="113" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B113" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C113" s="2"/>
       <c r="D113" s="2"/>
@@ -3207,19 +3247,19 @@
         <v>100000</v>
       </c>
       <c r="H113" s="16" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="I113" s="16" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="J113" s="16" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="K113" s="16"/>
     </row>
     <row r="114" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B114" s="2" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="C114" s="2"/>
       <c r="D114" s="2"/>
@@ -3229,16 +3269,16 @@
         <v>0.152</v>
       </c>
       <c r="H114" s="16" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="I114" s="16" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="J114" s="16" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="K114" s="16" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
   </sheetData>
@@ -3251,27 +3291,27 @@
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="B15:K15"/>
     <mergeCell ref="B17:K17"/>
-    <mergeCell ref="B29:F29"/>
     <mergeCell ref="B30:F30"/>
     <mergeCell ref="B31:F31"/>
     <mergeCell ref="B32:F32"/>
-    <mergeCell ref="B34:K34"/>
-    <mergeCell ref="B37:F37"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="B35:K35"/>
     <mergeCell ref="B38:F38"/>
     <mergeCell ref="B39:F39"/>
     <mergeCell ref="B40:F40"/>
-    <mergeCell ref="B42:K42"/>
-    <mergeCell ref="B45:F45"/>
+    <mergeCell ref="B41:F41"/>
+    <mergeCell ref="B43:K43"/>
     <mergeCell ref="B46:F46"/>
     <mergeCell ref="B47:F47"/>
     <mergeCell ref="B48:F48"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="B50:F50"/>
     <mergeCell ref="B51:F51"/>
-    <mergeCell ref="B53:K53"/>
-    <mergeCell ref="B54:F54"/>
+    <mergeCell ref="B52:F52"/>
+    <mergeCell ref="B54:K54"/>
     <mergeCell ref="B55:F55"/>
     <mergeCell ref="B56:F56"/>
+    <mergeCell ref="B57:F57"/>
     <mergeCell ref="B64:K64"/>
     <mergeCell ref="B65:K65"/>
     <mergeCell ref="B66:F66"/>

</xml_diff>

<commit_message>
Power budget: add ribbon output pull-down load, zip the spreadsheet
</commit_message>
<xml_diff>
--- a/docs/05-Power-Budget/Fill-A-Bot-Main-Control-Power-Budget.xlsx
+++ b/docs/05-Power-Budget/Fill-A-Bot-Main-Control-Power-Budget.xlsx
@@ -175,13 +175,13 @@
     <t xml:space="preserve">5.1V / 19.8k ohm = 0.258mA.</t>
   </si>
   <si>
-    <t xml:space="preserve">LCD E pull-down (while E is high)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100k ohm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.1V / 99k ohm = 0.052mA. Sourced by RC5.</t>
+    <t xml:space="preserve">100k pull-downs driven high: LCD E plus 4 ribbon outputs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100k ohm each (R24 here, 4 on teammates' boards)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each 5.1V / 99k ohm = 0.052mA. R24 on LCD E, plus the 100k pull-downs my 4 ribbon outputs drive on Clay's and Troy's boards.</t>
   </si>
   <si>
     <t xml:space="preserve">LCD contrast trimmer</t>
@@ -619,7 +619,7 @@
     <t xml:space="preserve">LCD E pull-down resistor</t>
   </si>
   <si>
-    <t xml:space="preserve">100k ohm from E to GND. Draws current only while RC5 drives E high.</t>
+    <t xml:space="preserve">100k ohm pull-downs: R24 on LCD E, and the pull-downs teammates put on their ribbon inputs. Draws current only while the line is high.</t>
   </si>
   <si>
     <t xml:space="preserve">Adapter cord and jack resistance, round trip</t>
@@ -1748,12 +1748,12 @@
         <v>1</v>
       </c>
       <c r="F25" s="8" t="n">
-        <f aca="false">ROUNDUP($G$72/($G$113*(1-$G$105))*1000,3)</f>
-        <v>0.052</v>
+        <f aca="false">5*ROUNDUP($G$72/($G$113*(1-$G$105))*1000,3)</f>
+        <v>0.26</v>
       </c>
       <c r="G25" s="8" t="n">
         <f aca="false">E25*F25</f>
-        <v>0.052</v>
+        <v>0.26</v>
       </c>
       <c r="H25" s="6" t="s">
         <v>18</v>
@@ -1899,7 +1899,7 @@
       <c r="F30" s="16"/>
       <c r="G30" s="12" t="n">
         <f aca="false">SUM(G19:G29)</f>
-        <v>345.606</v>
+        <v>345.814</v>
       </c>
       <c r="H30" s="17" t="s">
         <v>18</v>
@@ -1931,7 +1931,7 @@
       <c r="F32" s="16"/>
       <c r="G32" s="12" t="n">
         <f aca="false">ROUNDUP(G30*(1+G31),3)</f>
-        <v>432.008</v>
+        <v>432.268</v>
       </c>
       <c r="H32" s="17" t="s">
         <v>18</v>
@@ -1947,7 +1947,7 @@
       <c r="F33" s="3"/>
       <c r="G33" s="19" t="n">
         <f aca="false">G32*$G$70/1000</f>
-        <v>2.16004</v>
+        <v>2.16134</v>
       </c>
       <c r="H33" s="17" t="s">
         <v>70</v>
@@ -2042,7 +2042,7 @@
       <c r="F38" s="3"/>
       <c r="G38" s="19" t="n">
         <f aca="false">G32</f>
-        <v>432.008</v>
+        <v>432.268</v>
       </c>
       <c r="H38" s="17" t="s">
         <v>18</v>
@@ -2058,7 +2058,7 @@
       <c r="F39" s="16"/>
       <c r="G39" s="12" t="n">
         <f aca="false">G37-G38</f>
-        <v>1067.992</v>
+        <v>1067.732</v>
       </c>
       <c r="H39" s="17" t="s">
         <v>18</v>
@@ -2090,7 +2090,7 @@
       <c r="F41" s="16"/>
       <c r="G41" s="12" t="n">
         <f aca="false">G40-G32</f>
-        <v>787.992</v>
+        <v>787.732</v>
       </c>
       <c r="H41" s="17" t="s">
         <v>18</v>
@@ -2217,7 +2217,7 @@
       <c r="F48" s="3"/>
       <c r="G48" s="19" t="n">
         <f aca="false">G32</f>
-        <v>432.008</v>
+        <v>432.268</v>
       </c>
       <c r="H48" s="17" t="s">
         <v>18</v>
@@ -2280,7 +2280,7 @@
       <c r="F51" s="16"/>
       <c r="G51" s="12" t="n">
         <f aca="false">G48+G49+G50</f>
-        <v>444.039</v>
+        <v>444.299</v>
       </c>
       <c r="H51" s="17" t="s">
         <v>18</v>
@@ -2296,7 +2296,7 @@
       <c r="F52" s="16"/>
       <c r="G52" s="12" t="n">
         <f aca="false">G45-G51</f>
-        <v>1555.961</v>
+        <v>1555.701</v>
       </c>
       <c r="H52" s="17" t="s">
         <v>18</v>
@@ -2312,7 +2312,7 @@
       <c r="F53" s="3"/>
       <c r="G53" s="19" t="n">
         <f aca="false">E45*G51/1000</f>
-        <v>3.996351</v>
+        <v>3.998691</v>
       </c>
       <c r="H53" s="17" t="s">
         <v>70</v>
@@ -2602,7 +2602,7 @@
       <c r="F75" s="3"/>
       <c r="G75" s="19" t="n">
         <f aca="false">G69-G73/2-$G$114*G51/1000</f>
-        <v>8.407506072</v>
+        <v>8.407466552</v>
       </c>
       <c r="H75" s="17" t="s">
         <v>111</v>
@@ -2643,7 +2643,7 @@
       <c r="F77" s="16"/>
       <c r="G77" s="12" t="n">
         <f aca="false">G75-G76</f>
-        <v>1.807506072</v>
+        <v>1.807466552</v>
       </c>
       <c r="H77" s="17" t="s">
         <v>111</v>
@@ -2834,7 +2834,7 @@
       <c r="F86" s="3"/>
       <c r="G86" s="19" t="n">
         <f aca="false">(G68-G71)*G32/1000+G68*G49/1000</f>
-        <v>2.0601364</v>
+        <v>2.0613194</v>
       </c>
       <c r="H86" s="17" t="s">
         <v>70</v>
@@ -2853,7 +2853,7 @@
       <c r="F87" s="16"/>
       <c r="G87" s="23" t="n">
         <f aca="false">G79+G86*G83</f>
-        <v>70.902046</v>
+        <v>70.919791</v>
       </c>
       <c r="H87" s="17" t="s">
         <v>136</v>
@@ -2894,7 +2894,7 @@
       <c r="F89" s="16"/>
       <c r="G89" s="23" t="n">
         <f aca="false">G84-G87</f>
-        <v>54.097954</v>
+        <v>54.080209</v>
       </c>
       <c r="H89" s="17" t="s">
         <v>136</v>
@@ -2913,7 +2913,7 @@
       <c r="F90" s="3"/>
       <c r="G90" s="22" t="n">
         <f aca="false">G86*G82</f>
-        <v>20.601364</v>
+        <v>20.613194</v>
       </c>
       <c r="H90" s="17" t="s">
         <v>136</v>

</xml_diff>